<commit_message>
new terms from printed doc
</commit_message>
<xml_diff>
--- a/glossary.xlsx
+++ b/glossary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/SystemDocumentation/github/uactechdoc/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2730F25D-26C7-404C-B6F3-7D1E77C0C46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB7FCEA1-3E98-2449-ABA4-43BF03913242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{FD61D8A1-D7A7-6B4D-AB92-59721C5EF8F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="180">
   <si>
     <t>Topic</t>
   </si>
@@ -433,6 +433,150 @@
   <si>
     <t>A composite of multiple video sources (up to 4) into a single layered output with resizable, positioned boxes over a background. It’s ideal for picture-in-picture (PiP) layouts in live productions, such as news shows, conferences, or multi-camera streams. SuperSource excels for complex, preset-driven live layouts like news or conferences, while DVE offers flexibility for custom single-element effects or when stacking multiple keys.
 A SuperSource is itself a source</t>
+  </si>
+  <si>
+    <t>Barn Doors</t>
+  </si>
+  <si>
+    <t>Snoots, Snouts</t>
+  </si>
+  <si>
+    <t>Black hinged panels or shutters (which open and close like real barn doors) attached to the front of a lamp fixture to control the spread of the light beam. Also see Snoots (or Snouts) .</t>
+  </si>
+  <si>
+    <t>Scoop: See Flood,</t>
+  </si>
+  <si>
+    <t>Broad</t>
+  </si>
+  <si>
+    <t>A type of floodlight used to provide broadside flat lighting. When it has twin lamps, it is termed a double broad or broadside.</t>
+  </si>
+  <si>
+    <t>Century Stand</t>
+  </si>
+  <si>
+    <t>Upright, pole-like stand with clamps. It may be used to hold a gobo extra small lights etc</t>
+  </si>
+  <si>
+    <t>Junior</t>
+  </si>
+  <si>
+    <t>Deuce</t>
+  </si>
+  <si>
+    <t>Nickname for a 2-kW lamp. Also see Junior.</t>
+  </si>
+  <si>
+    <t>Dimmer Board</t>
+  </si>
+  <si>
+    <t>Houses the appropriate switches and controls for fading down and brightening lights or banks of lights.</t>
+  </si>
+  <si>
+    <t>Elbows</t>
+  </si>
+  <si>
+    <t>Special hooks used to keep cables off floors.</t>
+  </si>
+  <si>
+    <t>Flag</t>
+  </si>
+  <si>
+    <t>Small rectangular gobo. An even smaller gobo is termed a clip. Terminology is quite fluid here; a thin flag might be called a blade; a round one might be called a target or (if very small) a dot. A flag with a small hole is called an ear.</t>
+  </si>
+  <si>
+    <t>Flood</t>
+  </si>
+  <si>
+    <t>Floodlighting and spotlighting are the two basic types of lighting. The flood is designed to illuminate a broad expanse; it is also called a SCOOP.</t>
+  </si>
+  <si>
+    <t>Black screen, cloth, or sheet used to block off unwanted light reflections into the camera lens. Also applied to a built-in pattern projector for Lekolights</t>
+  </si>
+  <si>
+    <t>Inky</t>
+  </si>
+  <si>
+    <t>Baby spotlight usually mounted on the front of a camera to lend extra sparkle to a person's eyes and teeth. Originally this term was a contraction of "incandescent" (thus, a small incandescent spotlight), but it also is applied in current usage to a small spotlight using the newer quartz-iodine lamp.</t>
+  </si>
+  <si>
+    <t>A light not quite as bright as a senior, usually rated at one or two kilowatts.</t>
+  </si>
+  <si>
+    <t>Keg Light</t>
+  </si>
+  <si>
+    <t>Small spotlight in a housing that resembles a keg.</t>
+  </si>
+  <si>
+    <t>Klieg Light</t>
+  </si>
+  <si>
+    <t>A flood-spotlight (either way). (Trade name of Kliegl Bros. Lighting.)</t>
+  </si>
+  <si>
+    <t>Leko</t>
+  </si>
+  <si>
+    <t>Leko (Lekolite): Special spotlight shuttered to provide a desired pattern of light. (Trade name of Century Lighting, Inc.)</t>
+  </si>
+  <si>
+    <t>Luninaire</t>
+  </si>
+  <si>
+    <t>Light fixture with lamp. (General term.)</t>
+  </si>
+  <si>
+    <t>Reflectors</t>
+  </si>
+  <si>
+    <t>Brightly polished concave surfaces used behind a lamp to concentrate the light rays in one direction. The term is also applied to exterior sheets (up to about 6' X 6') used to reflect light into desired locations (such as shadow fill).</t>
+  </si>
+  <si>
+    <t>Rifle</t>
+  </si>
+  <si>
+    <t>Spotlight with a very small beam of light used to pinpoint a small detail.</t>
+  </si>
+  <si>
+    <t>Scoop</t>
+  </si>
+  <si>
+    <t>Snoot</t>
+  </si>
+  <si>
+    <t>Snoots (or Snouts): Hoods placed in front of lamp housings to limit the area illuminated.</t>
+  </si>
+  <si>
+    <t>Spiders</t>
+  </si>
+  <si>
+    <t>The points where cables converge for connection to the current main. They are so termed because they resemble a spider's web.</t>
+  </si>
+  <si>
+    <t>Spill</t>
+  </si>
+  <si>
+    <t>Term for excess light that falls in areas not intended</t>
+  </si>
+  <si>
+    <t>Spotlight</t>
+  </si>
+  <si>
+    <t>Highly concentrated beam of light.</t>
+  </si>
+  <si>
+    <t>Striplights</t>
+  </si>
+  <si>
+    <t>Lights arranged in strips for lighting backings, windows, and cycloramas ("cycs"). A cyclorama is a semicircular or U-shaped hanging for a background.</t>
+  </si>
+  <si>
+    <t>Teaser</t>
+  </si>
+  <si>
+    <t>Large, flat gobo used to block overhead back light from the camera lens</t>
   </si>
 </sst>
 </file>
@@ -510,8 +654,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}" name="Table1" displayName="Table1" ref="A1:D60" totalsRowShown="0" dataDxfId="4">
-  <autoFilter ref="A1:D60" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}" name="Table1" displayName="Table1" ref="A1:D84" totalsRowShown="0" dataDxfId="4">
+  <autoFilter ref="A1:D84" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D56">
     <sortCondition ref="A2:A56"/>
     <sortCondition ref="B2:B56"/>
@@ -823,10 +967,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{327B4C12-DB51-F04E-97D5-67343BD74C6D}">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="94.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1574,6 +1719,300 @@
       </c>
       <c r="D60" s="2" t="s">
         <v>130</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C62" s="1"/>
+      <c r="D62" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C63" s="1"/>
+      <c r="D63" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C65" s="1"/>
+      <c r="D65" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C66" s="1"/>
+      <c r="D66" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C67" s="1"/>
+      <c r="D67" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C68" s="1"/>
+      <c r="D68" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C69" s="1"/>
+      <c r="D69" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C70" s="1"/>
+      <c r="D70" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C71" s="1"/>
+      <c r="D71" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C72" s="1"/>
+      <c r="D72" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C73" s="1"/>
+      <c r="D73" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C74" s="1"/>
+      <c r="D74" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C75" s="1"/>
+      <c r="D75" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C76" s="1"/>
+      <c r="D76" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C77" s="1"/>
+      <c r="D77" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C79" s="1"/>
+      <c r="D79" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C80" s="1"/>
+      <c r="D80" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C81" s="1"/>
+      <c r="D81" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C82" s="1"/>
+      <c r="D82" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C83" s="1"/>
+      <c r="D83" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C84" s="1"/>
+      <c r="D84" s="2" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added numerous lighting terms
</commit_message>
<xml_diff>
--- a/glossary.xlsx
+++ b/glossary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB7FCEA1-3E98-2449-ABA4-43BF03913242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06DC177A-AAC5-A246-9E9E-1180E16C9235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{FD61D8A1-D7A7-6B4D-AB92-59721C5EF8F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="279">
   <si>
     <t>Topic</t>
   </si>
@@ -101,21 +101,9 @@
     <t>Dimmer</t>
   </si>
   <si>
-    <t>: A device which regulates the power sent to a lighting instrument (typically incandescent) this allows the intensity of the instrument to be varied. Usually DMX controlled, but could be controlled via an analog or proprietary protocols.</t>
-  </si>
-  <si>
-    <t>DMX / DMX512</t>
-  </si>
-  <si>
-    <t xml:space="preserve">: an industry standard lighting control protocol. A universe is a group of 512 addresses, numbered 1 through 512. See also RDM. </t>
-  </si>
-  <si>
     <t>Gel</t>
   </si>
   <si>
-    <t xml:space="preserve">: a coloured sheet of special plastic which is used to physically change the colour of a light. </t>
-  </si>
-  <si>
     <t>Gel Frame</t>
   </si>
   <si>
@@ -143,13 +131,7 @@
     <t>Par / Par Can</t>
   </si>
   <si>
-    <t>: a type of lighting instrument with a fixed beam width. Some of them look like paint cans. Generally used for washes.</t>
-  </si>
-  <si>
     <t>RDM / Remote Device Management</t>
-  </si>
-  <si>
-    <t>: This is a management protocol that can run over the same cables as DMX. It is a bi-directional protocol. It can be used to change the configuration of some lighting fixtures (such as our ETC fixtures) without having physical access to the fixture.</t>
   </si>
   <si>
     <t>Rotator</t>
@@ -492,9 +474,6 @@
     <t>Floodlighting and spotlighting are the two basic types of lighting. The flood is designed to illuminate a broad expanse; it is also called a SCOOP.</t>
   </si>
   <si>
-    <t>Black screen, cloth, or sheet used to block off unwanted light reflections into the camera lens. Also applied to a built-in pattern projector for Lekolights</t>
-  </si>
-  <si>
     <t>Inky</t>
   </si>
   <si>
@@ -577,6 +556,422 @@
   </si>
   <si>
     <t>Large, flat gobo used to block overhead back light from the camera lens</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - The state of being able to see or be seen. The most important fundamental. If
+the audience can’t see, everything else the lighting designer does is a waste of time.
+Studies have shown that visibility affects our ability to understand spoken speech. This
+doesn’t mean the audience must see everything all the time, but they should be focused
+on what the story is telling us.</t>
+  </si>
+  <si>
+    <t>Visibility</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - The strength or amount of light produced by a specific lamp source. It is not
+always about how ‘bright’ the light is, but how ‘dim’.</t>
+  </si>
+  <si>
+    <t>Intensity</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Where the light hits and from what angle. Careful consideration of these
+factors can determine the visibility of the actor, depth and detail of scenery, as well as
+other areas such as given circumstances and mood.</t>
+  </si>
+  <si>
+    <t>Distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - The use of color is one of the most noticeable defining elements of any lighting
+design. For many designers, color is the most personal of elements, and often times not
+only defines the design, but the personal style of the designer.</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>– Any change in visibility, intensity, distribution, or color, as well as physical
+movement when using Moving Lights. Not as apparent as some of the others, this is still
+a very important element that has a significant effect on the lighting design.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Movement </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – When an object or performer moves in and out of light.</t>
+  </si>
+  <si>
+    <t>Apparent Movement</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - When the light itself moves.</t>
+  </si>
+  <si>
+    <t>Actual Movement</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – The trigger for an action to be carried out at a specific time, normally called by a
+stage manager. They can be necessary for a lighting change or effect, a sound effect, or
+some sort of stage or set movement/change.</t>
+  </si>
+  <si>
+    <t>Cue</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – A document like an architectural blueprint used specifically by theatrical
+lighting designers to illustrate and communicate the lighting design to members of the
+crew and staff.</t>
+  </si>
+  <si>
+    <t>Lightplot</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – The range of frequencies of electromagnetic radiation.
+Includes all visible and invisible light, radio and television signals, x-rays and microwaves.</t>
+  </si>
+  <si>
+    <t>Electromagnetic Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Lighting fixture that can be used to create a general "fill" of light and
+color evenly across the stage.</t>
+  </si>
+  <si>
+    <t>Wash Fixture</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Fixture with a hard-edged beam. These fixtures are best for creating a
+“special” or using light to mask off a small, precise area, and also are the fixtures to use if
+you want to project a pattern, or “gobo”.</t>
+  </si>
+  <si>
+    <t>Spot Fixture</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - The most commonly known instrument. Follow spots are used to highlight
+and follow a single performer onstage. Spotlights are controlled by a spotlight operator
+(or Spot Op) who tracks actors around the stage. Follow spots require a certain amount
+of skill to operate smoothly. They typically have a variety of colors that can be inserted
+with the flip of a lever, as well as a gate, dowser, focus control, and an iris. Used to
+follow a lead talent on stage.</t>
+  </si>
+  <si>
+    <t>Follow Spot</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - A small, stenciled, circular disc used in lighting fixtures to create a
+projected image or pattern. The term Gobo is short for “Go Between Optics”, describing
+the location where it needs to be positioned in the light path of a lighting fixture.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – The point at which light waves intersect after refraction or reflection.</t>
+  </si>
+  <si>
+    <t>Focal Point</t>
+  </si>
+  <si>
+    <t>PAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Pronounced freh-NEL - A Fresnel lens maintains the curvature and prescription
+of a large convex lens in a much thinner version. The curve of the lens is stepped back
+towards the flat side at regular intervals. This is less expensive to produce and allows
+more even heat distribution through the glass, protecting the lens from expansion and
+contraction. The trade-off is a fuzzier, softer field. Used often for top light, backlight, and
+general washes.</t>
+  </si>
+  <si>
+    <t>Fresnel</t>
+  </si>
+  <si>
+    <t>Cyclorama</t>
+  </si>
+  <si>
+    <t>Cyc Lights</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Light from the back of a performer or object. Often used to pull the subject
+away from the background, sculps and adds depth to the subject. In film this can be
+referred to a hair light.</t>
+  </si>
+  <si>
+    <t>Back Light</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Light from up above or at the height of the subject to help sculpt the body
+and add fill to the sides of the subject. In film this is referred to as fill light.</t>
+  </si>
+  <si>
+    <t>Side Light</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Light directly above the subject.</t>
+  </si>
+  <si>
+    <t>Top Light</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Light to the front of the subject.</t>
+  </si>
+  <si>
+    <t>Front Light</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - A method of lighting using a front light in conjunction with
+two side lights.</t>
+  </si>
+  <si>
+    <t>Three Point Lighting</t>
+  </si>
+  <si>
+    <t>– A method of lighting similar to Three Point Lighting using a front
+light, two side lights, and a backlight or using a front light, a fill light, a backlight, and w a
+background light that illuminates walls or other scenery around the subject.</t>
+  </si>
+  <si>
+    <t>Four Point Lighting</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – This method is widely known and used by theatre professionals.
+It uses two front lights at a 45-degree angle of the subject, one side being a warm gel
+color and the other side being a cool gel color. This helps replicate a highlight and
+shadow contrast with lighting.</t>
+  </si>
+  <si>
+    <t>McCandless Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Generally, a system of rope lines, blocks (pulleys), counterweights and
+related devices within a theater that enables a stage crew to fly (hoist) quickly, quietly
+and safely components such as curtains, lights, scenery, stage effects and, sometimes,
+people. These systems can either be manually operated or motorized. Rigging can also be
+stationary, or dead hung, in the case of an overhead grid.</t>
+  </si>
+  <si>
+    <t>Stage Rigging</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Originally a vertical pipe in a seating box used for stage lights, but now used
+to indicate any side lighting position.</t>
+  </si>
+  <si>
+    <t>Box Boom</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - An elevated service platform from which many of the technical functions of
+a theater, such as lighting and sound, may be manipulated.</t>
+  </si>
+  <si>
+    <t>Catwalk</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - The line set is the fundamental machine of a typical fly system. The function
+of a typical line set is to fly (raise and lower) a slender beam (typically a steel pipe) known
+as a batten by hoisting it with lift lines (typically synthetic rope or steel cable). By
+hanging scenery, lighting, or other equipment on a batten, they in turn may also be
+flown. A batten is said to be "flying in" when it is being lowered toward the stage, and
+"flying out" when it is being raised into the fly space. Battens may be just a few feet in
+length or may extend from one wing (side) of the stage to the other. A batten is
+suspended from above by at least two lift lines, but long battens may require six or more
+lift lines.</t>
+  </si>
+  <si>
+    <t>Line Sets</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - The means by which an instrument is connected to a dimmer or patch panel.
+Numbered for reference.</t>
+  </si>
+  <si>
+    <t>Circuit</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Method of flying scenery which uses a cradle containing
+weights to counterbalance the weight of flown scenery.</t>
+  </si>
+  <si>
+    <t>Counterweight System</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Part of the load in a counterweight system representing the weight of the
+empty batten; pipe weight should be left on the arbor when the load and its
+counterweight is removed.</t>
+  </si>
+  <si>
+    <t>Pipe Weight</t>
+  </si>
+  <si>
+    <t>Dimmer Rack</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - The room backstage which contains the dimmer racks which power the
+lighting rig in the theatre.</t>
+  </si>
+  <si>
+    <t>Dimmer Room</t>
+  </si>
+  <si>
+    <t>DMX</t>
+  </si>
+  <si>
+    <t>DMX Universe</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - An electronic device used in theatrical lighting design to control
+multiple lights at once, also known as a Light Board.</t>
+  </si>
+  <si>
+    <t>Lighting Console</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Ellipsoidal reflector spotlights do a lot and can be very precise. They can
+accept gobos and irises and have built-in shutters for shaping the field of light.
+Ellipsoidals require a degree of maintenance and finesse; they are less easy to use than
+other types of instruments and are a bit more expensive. Used often for front light or side
+light in dance.</t>
+  </si>
+  <si>
+    <t>Ellipsoidal</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - An ellipsoidal reflector spotlight (ERS) used in stage lighting.</t>
+  </si>
+  <si>
+    <t>Source Four</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Fixed at two points to the sides of the instrument, providing an axis of rotation.
+The base of the yoke is typically a single bolt around which the yoke can be rotated,
+providing a second axis of rotation. Combined together, these two axes allow the fixture
+to point nearly anywhere in a spherical range of motion encircling the yoke.</t>
+  </si>
+  <si>
+    <t>Yoke</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Cable or chain to be attached between the fixture and its truss. Lighting
+fixtures often are suspended very high above performers heads and could cause serious
+injury or death if they fell by accident or due to incorrect attachment. The safety cable
+would halt the fall of the fixture before it could cause serious damage or injury.</t>
+  </si>
+  <si>
+    <t>Safety Cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – A preliminary or advance focus. If you know where the light will be focused,
+point it in that general directions to make sure it is tight, and the cable will reach.
+Accessory Slot – On a Source Four, can hold multiple accessories for the light such as
+templates or template rotators.</t>
+  </si>
+  <si>
+    <t>Pre-focus</t>
+  </si>
+  <si>
+    <t>Gel or Light Filter</t>
+  </si>
+  <si>
+    <t>Gobo or Template</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - A color magazine or "boomerang" consisting of several gel frames which
+can be swung in front of the beam.</t>
+  </si>
+  <si>
+    <t>Boomerang</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - A metal flag used in larger follow spots and projection equipment to cut off the
+light beam without cutting off the electrical supply. Discharge lamps cannot be dimmed,
+so this is the only way of stopping light. Discharge lamps need a period of cooling down
+when they are turned off before they can be turned on again, so they should not be
+switched off if needed again within about two hours.</t>
+  </si>
+  <si>
+    <t>Douser</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Two horizontal masking shutters used in follow spots to shape the
+beam above and below.</t>
+  </si>
+  <si>
+    <t>Gate or Choppers</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Adjustable aperture which, when placed in the gate of a profile lantern, varies the
+size of a beam of light. Originally, iris diaphragm. Most follow spots have an iris
+permanently installed.</t>
+  </si>
+  <si>
+    <t>Iris</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – Cyc for short. A background device employed to cover the back and
+sometimes the sides of the stage and used with special lighting to create the illusion of
+sky, open space, or great distance at the rear of the stage setting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - To reduce the beam size of a Fresnel by moving the lamp further from the lens.</t>
+  </si>
+  <si>
+    <t>Spot</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Remotely controllable "intelligent" lighting instrument.
+Each instrument is capable of a massive variety of effects which are operated live via a
+moving light control desk or can be pre-programmed by a standard memory lighting
+desk. The instruments require a power supply and a data cable (normally carrying
+DMX512 signal from the control desk).</t>
+  </si>
+  <si>
+    <t>Moving Head or Moving Light</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> – A metal blade which can be used to shape the edge of the beam of light.
+Shutters (normally four) are located in the gate at the center of the light. The position of
+a shutter in the light beam is known as the shutter cut.</t>
+  </si>
+  <si>
+    <t>Shutters</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - An instrument specially designed for lighting cycloramas. They serve one of
+the same functions as a strip light. Their reflector, however, shapes the field in such a
+way that the cyc is illuminated as brightly at the bottom as it is at the top.  Used often to light a cyclorama, backdrop or background.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - </t>
+  </si>
+  <si>
+    <t>Electrical or electronic device that controls the amount of electricity passed to
+a lamp, and therefore the intensity of the lamp.  A device which regulates the power sent to a lighting instrument (typically incandescent) this allows the intensity of the instrument to be varied. Usually DMX controlled, but could be controlled via an analog or proprietary protocols.</t>
+  </si>
+  <si>
+    <t>A number of individual dimmer circuits mounted in a cabinet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMX (Digital Multiplex) - The standard digital communication protocol that is used to
+remotely control dimmer rack and intelligent lighting fixtures. An industry standard lighting control protocol. A universe is a group of 512 addresses, numbered 1 through 512. See also RDM. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A set of channels, 512 to be precise, on which DMX signals operate.</t>
+  </si>
+  <si>
+    <t>: a coloured sheet of special plastic which is used to physically change the colour of a light. A transparent colored material that is used in theater, event production, photography, videography and cinematography to color light and for color correction.</t>
+  </si>
+  <si>
+    <t>(Parabolic aluminized reflector) - Short for parabolic aluminized reflectors. These
+lights throw a bright hazy beam in the shape of an oval or parabola. The body of a PAR-can is nothing but a
+metal shell for the lamp, which includes a lens and reflector within it. A PAR lamp is a lot
+like a car headlight. By putting different versions of the lamp into the instrument, the
+beam can be wide, medium, narrow, or very narrow. Used often for back light or stage
+wash.</t>
+  </si>
+  <si>
+    <t>A type of lighting instrument with a fixed beam width. Some of them look like paint cans. Generally used for washes.</t>
+  </si>
+  <si>
+    <t>This is a management protocol that can run over the same cables as DMX. It is a bi-directional protocol. It can be used to change the configuration of some lighting fixtures (such as our ETC fixtures) without having physical access to the fixture.</t>
   </si>
 </sst>
 </file>
@@ -654,11 +1049,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}" name="Table1" displayName="Table1" ref="A1:D84" totalsRowShown="0" dataDxfId="4">
-  <autoFilter ref="A1:D84" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D56">
-    <sortCondition ref="A2:A56"/>
-    <sortCondition ref="B2:B56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}" name="Table1" displayName="Table1" ref="A1:D133" totalsRowShown="0" dataDxfId="4">
+  <autoFilter ref="A1:D133" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D133">
+    <sortCondition ref="A2:A133"/>
+    <sortCondition ref="B2:B133"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{A991846A-4384-6048-992B-FAECE1424BD1}" name="Topic" dataDxfId="3"/>
@@ -967,7 +1362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{327B4C12-DB51-F04E-97D5-67343BD74C6D}">
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -991,1028 +1386,1616 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="68" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>46</v>
+        <v>186</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>18</v>
+        <v>184</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="2" t="s">
-        <v>19</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>20</v>
+        <v>208</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="2" t="s">
-        <v>21</v>
+        <v>207</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="1"/>
+        <v>126</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>127</v>
+      </c>
       <c r="D20" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>24</v>
+        <v>255</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>26</v>
+        <v>224</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="2" t="s">
-        <v>27</v>
+        <v>223</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>28</v>
+        <v>130</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="2" t="s">
-        <v>29</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>30</v>
+        <v>226</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>32</v>
+        <v>132</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>36</v>
+        <v>230</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>38</v>
+        <v>180</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>50</v>
+        <v>232</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>52</v>
+        <v>188</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="68" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>206</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>40</v>
+        <v>205</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="2" t="s">
-        <v>41</v>
+        <v>262</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>95</v>
+        <v>36</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" s="1"/>
+        <v>135</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>134</v>
+      </c>
       <c r="D33" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="68" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>95</v>
+        <v>36</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>108</v>
+        <v>137</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>101</v>
+        <v>235</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="2" t="s">
-        <v>103</v>
+        <v>272</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>102</v>
+        <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>105</v>
+        <v>237</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>102</v>
+        <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>118</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="C39" s="1"/>
       <c r="D39" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>117</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="C40" s="1"/>
       <c r="D40" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>116</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="C41" s="1"/>
       <c r="D41" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>115</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="C42" s="1"/>
       <c r="D42" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>56</v>
+        <v>192</v>
       </c>
       <c r="C43" s="1"/>
       <c r="D43" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>60</v>
+        <v>243</v>
       </c>
       <c r="C44" s="1"/>
       <c r="D44" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>5</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="C45" s="1"/>
       <c r="D45" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>4</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="C46" s="1"/>
       <c r="D46" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>61</v>
+        <v>201</v>
       </c>
       <c r="C47" s="1"/>
       <c r="D47" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="102" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>11</v>
+        <v>198</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>12</v>
+        <v>218</v>
       </c>
       <c r="C49" s="1"/>
       <c r="D49" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="102" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>8</v>
+        <v>204</v>
       </c>
       <c r="C50" s="1"/>
       <c r="D50" s="2" t="s">
-        <v>15</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>97</v>
+        <v>214</v>
       </c>
       <c r="C51" s="1"/>
       <c r="D51" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>92</v>
+        <v>259</v>
       </c>
       <c r="C52" s="1"/>
       <c r="D52" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>91</v>
+        <v>22</v>
       </c>
       <c r="C54" s="1"/>
       <c r="D54" s="2" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>9</v>
+        <v>252</v>
       </c>
       <c r="C55" s="1"/>
       <c r="D55" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C56" s="1"/>
       <c r="D56" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>123</v>
+        <v>253</v>
       </c>
       <c r="C57" s="1"/>
       <c r="D57" s="2" t="s">
-        <v>124</v>
+        <v>199</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>126</v>
+        <v>26</v>
       </c>
       <c r="C58" s="1"/>
       <c r="D58" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>128</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="C59" s="1"/>
       <c r="D59" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>129</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="C60" s="1"/>
       <c r="D60" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>133</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="C61" s="1"/>
       <c r="D61" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A62" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="C62" s="1"/>
       <c r="D62" s="2" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="C63" s="1"/>
       <c r="D63" s="2" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>140</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="C64" s="1"/>
       <c r="D64" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="C65" s="1"/>
       <c r="D65" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C66" s="1"/>
       <c r="D66" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>147</v>
+        <v>241</v>
       </c>
       <c r="C67" s="1"/>
       <c r="D67" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>149</v>
+        <v>190</v>
       </c>
       <c r="C68" s="1"/>
       <c r="D68" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="153" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>28</v>
+        <v>228</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C70" s="1"/>
       <c r="D70" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="68" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>140</v>
+        <v>220</v>
       </c>
       <c r="C71" s="1"/>
       <c r="D71" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>155</v>
+        <v>182</v>
       </c>
       <c r="C72" s="1"/>
       <c r="D72" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>157</v>
+        <v>266</v>
       </c>
       <c r="C73" s="1"/>
       <c r="D73" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="102" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>159</v>
+        <v>202</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>161</v>
+        <v>30</v>
       </c>
       <c r="C75" s="1"/>
       <c r="D75" s="2" t="s">
-        <v>162</v>
+        <v>277</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>163</v>
+        <v>234</v>
       </c>
       <c r="C76" s="1"/>
       <c r="D76" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="68" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>165</v>
+        <v>251</v>
       </c>
       <c r="C77" s="1"/>
       <c r="D77" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>149</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="C78" s="1"/>
       <c r="D78" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="C79" s="1"/>
       <c r="D79" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="C80" s="1"/>
       <c r="D80" s="2" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>172</v>
+        <v>32</v>
       </c>
       <c r="C81" s="1"/>
       <c r="D81" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="68" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>174</v>
+        <v>249</v>
       </c>
       <c r="C82" s="1"/>
       <c r="D82" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>176</v>
+        <v>44</v>
       </c>
       <c r="C83" s="1"/>
       <c r="D83" s="2" t="s">
-        <v>177</v>
+        <v>47</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="C84" s="1"/>
+        <v>160</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>143</v>
+      </c>
       <c r="D84" s="2" t="s">
-        <v>179</v>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C85" s="1"/>
+      <c r="D85" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C86" s="1"/>
+      <c r="D86" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C87" s="1"/>
+      <c r="D87" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C88" s="1"/>
+      <c r="D88" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C89" s="1"/>
+      <c r="D89" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C90" s="1"/>
+      <c r="D90" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C91" s="1"/>
+      <c r="D91" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C92" s="1"/>
+      <c r="D92" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C93" s="1"/>
+      <c r="D93" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C94" s="1"/>
+      <c r="D94" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C95" s="1"/>
+      <c r="D95" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C96" s="1"/>
+      <c r="D96" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C97" s="1"/>
+      <c r="D97" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C98" s="1"/>
+      <c r="D98" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C99" s="1"/>
+      <c r="D99" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C100" s="1"/>
+      <c r="D100" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C101" s="1"/>
+      <c r="D101" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C102" s="1"/>
+      <c r="D102" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C103" s="1"/>
+      <c r="D103" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C104" s="1"/>
+      <c r="D104" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C105" s="1"/>
+      <c r="D105" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C106" s="1"/>
+      <c r="D106" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C107" s="1"/>
+      <c r="D107" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C110" s="1"/>
+      <c r="D110" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C113" s="1"/>
+      <c r="D113" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A114" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C114" s="1"/>
+      <c r="D114" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C115" s="1"/>
+      <c r="D115" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C116" s="1"/>
+      <c r="D116" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A117" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A118" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C119" s="1"/>
+      <c r="D119" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C120" s="1"/>
+      <c r="D120" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A121" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C121" s="1"/>
+      <c r="D121" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A122" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C122" s="1"/>
+      <c r="D122" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A123" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C123" s="1"/>
+      <c r="D123" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A124" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C124" s="1"/>
+      <c r="D124" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A125" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A126" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C126" s="1"/>
+      <c r="D126" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A127" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C127" s="1"/>
+      <c r="D127" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A128" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C128" s="1"/>
+      <c r="D128" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A129" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C129" s="1"/>
+      <c r="D129" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C130" s="1"/>
+      <c r="D130" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A131" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A132" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C132" s="1"/>
+      <c r="D132" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A133" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C133" s="1"/>
+      <c r="D133" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added some power terms
</commit_message>
<xml_diff>
--- a/glossary.xlsx
+++ b/glossary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3B644F-109A-DD44-B5E3-DADBE89512D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{105215B6-4183-FA44-891E-21F40F93D067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{FD61D8A1-D7A7-6B4D-AB92-59721C5EF8F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="333">
   <si>
     <t>Topic</t>
   </si>
@@ -294,9 +294,6 @@
   </si>
   <si>
     <t>This is a heavy duty 20 Amp  connector with circular locking contacts  (hence the **L** in the name). There is an *R* and a *P* suffix for the *recepacle* and *plug*.</t>
-  </si>
-  <si>
-    <t>This is a regular three-prong   connector  good for 15 Amps . There is an *R* and a *P* suffix for the *recepacle* and *plug*.</t>
   </si>
   <si>
     <t>Nema 5-15</t>
@@ -1119,6 +1116,24 @@
 The base of the yoke is typically a single bolt around which the yoke can be rotated,
 providing a second axis of rotation. Combined together, these two axes allow the fixture
 to point nearly anywhere in a spherical range of motion encircling the yoke.</t>
+  </si>
+  <si>
+    <t>Nema 1-15</t>
+  </si>
+  <si>
+    <t>This is a regular two-prong  connector good for 15 Amps . There is an *R* and a *P* suffix for the *recepacle* and *plug*.</t>
+  </si>
+  <si>
+    <t>This is a regular three-prong connector good for 15 Amps . There is an *R* and a *P* suffix for the *recepacle* and *plug*.</t>
+  </si>
+  <si>
+    <t>Nema 5-15, Nema 6-20</t>
+  </si>
+  <si>
+    <t>Nema 1-15, Nema 6-20</t>
+  </si>
+  <si>
+    <t>Nema 1-15, Nema 5-15</t>
   </si>
 </sst>
 </file>
@@ -1168,13 +1183,13 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1199,17 +1214,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}" name="Table1" displayName="Table1" ref="A1:E158" totalsRowShown="0" dataDxfId="5">
-  <autoFilter ref="A1:E158" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E158">
-    <sortCondition ref="B1:B158"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}" name="Table1" displayName="Table1" ref="A1:E159" totalsRowShown="0" dataDxfId="5">
+  <autoFilter ref="A1:E159" xr:uid="{314A4941-A8BA-2346-8EA0-5892B4F1C3B7}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E159">
+    <sortCondition ref="B1:B159"/>
   </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{A991846A-4384-6048-992B-FAECE1424BD1}" name="Topic" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{ABA7B585-B679-4046-A73C-5497CC96B4A8}" name="Term" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{BCC184D7-6C8F-B940-B216-AB00E086E8CE}" name="Sense" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{01E09C02-E371-8D42-9078-8A75C09E6982}" name="SeeAlso" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{A2D271FE-F834-0142-AB0D-F732DE4B8C76}" name="Definition" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{BCC184D7-6C8F-B940-B216-AB00E086E8CE}" name="Sense" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{01E09C02-E371-8D42-9078-8A75C09E6982}" name="SeeAlso" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{A2D271FE-F834-0142-AB0D-F732DE4B8C76}" name="Definition" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1512,11 +1527,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{327B4C12-DB51-F04E-97D5-67343BD74C6D}">
-  <dimension ref="A1:E158"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.5" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="94.33203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1529,7 +1544,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -1543,14 +1558,14 @@
         <v>29</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1558,14 +1573,14 @@
         <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1603,14 +1618,14 @@
         <v>28</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -1618,14 +1633,14 @@
         <v>28</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C7" s="1">
         <v>1</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -1633,14 +1648,14 @@
         <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1648,16 +1663,16 @@
         <v>28</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C9" s="1">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1665,14 +1680,14 @@
         <v>28</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C10" s="1">
         <v>1</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1680,14 +1695,14 @@
         <v>28</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C11" s="1">
         <v>1</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1695,14 +1710,14 @@
         <v>28</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C12" s="1">
         <v>1</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1710,14 +1725,14 @@
         <v>14</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C13" s="1">
         <v>1</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1755,14 +1770,14 @@
         <v>82</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1777,7 +1792,7 @@
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1785,14 +1800,14 @@
         <v>28</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C18" s="1">
         <v>1</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1800,14 +1815,14 @@
         <v>28</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C19" s="1">
         <v>1</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1821,7 +1836,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>57</v>
@@ -1839,7 +1854,7 @@
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1847,14 +1862,14 @@
         <v>28</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C22" s="1">
         <v>1</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -1862,14 +1877,14 @@
         <v>28</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C23" s="1">
         <v>1</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -1892,14 +1907,14 @@
         <v>28</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C25" s="1">
         <v>1</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -1907,14 +1922,14 @@
         <v>28</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C26" s="1">
         <v>1</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1922,14 +1937,14 @@
         <v>28</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C27" s="1">
         <v>2</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -1937,14 +1952,14 @@
         <v>28</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C28" s="1">
         <v>1</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -1952,14 +1967,14 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C29" s="1">
         <v>1</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1967,7 +1982,7 @@
         <v>54</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C30" s="1">
         <v>1</v>
@@ -1976,7 +1991,7 @@
         <v>76</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2016,16 +2031,16 @@
         <v>28</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" s="1">
+        <v>1</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="C33" s="1">
-        <v>1</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -2040,7 +2055,7 @@
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2048,14 +2063,14 @@
         <v>28</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C35" s="1">
         <v>1</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2063,14 +2078,14 @@
         <v>28</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C36" s="1">
         <v>1</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2078,14 +2093,14 @@
         <v>28</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C37" s="1">
         <v>1</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -2108,14 +2123,14 @@
         <v>28</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C39" s="1">
         <v>1</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2123,14 +2138,16 @@
         <v>28</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C40" s="1">
         <v>1</v>
       </c>
-      <c r="D40" s="1"/>
+      <c r="D40" s="1" t="s">
+        <v>268</v>
+      </c>
       <c r="E40" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -2138,14 +2155,14 @@
         <v>28</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C41" s="1">
         <v>2</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2153,14 +2170,14 @@
         <v>28</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C42" s="1">
         <v>1</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -2168,14 +2185,14 @@
         <v>28</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C43" s="1">
         <v>1</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2198,16 +2215,16 @@
         <v>14</v>
       </c>
       <c r="B45" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C45" s="1">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C45" s="1">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2215,14 +2232,14 @@
         <v>28</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C46" s="1">
         <v>1</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2230,14 +2247,14 @@
         <v>28</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C47" s="1">
         <v>1</v>
       </c>
       <c r="D47" s="1"/>
       <c r="E47" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -2245,14 +2262,14 @@
         <v>28</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C48" s="1">
         <v>1</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2277,14 +2294,14 @@
         <v>28</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C50" s="1">
         <v>1</v>
       </c>
       <c r="D50" s="1"/>
       <c r="E50" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -2292,14 +2309,14 @@
         <v>28</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C51" s="1">
         <v>1</v>
       </c>
       <c r="D51" s="1"/>
       <c r="E51" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2307,14 +2324,14 @@
         <v>28</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C52" s="1">
         <v>1</v>
       </c>
       <c r="D52" s="1"/>
       <c r="E52" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2322,14 +2339,14 @@
         <v>28</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C53" s="1">
         <v>1</v>
       </c>
       <c r="D53" s="1"/>
       <c r="E53" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2337,14 +2354,14 @@
         <v>28</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C54" s="1">
         <v>1</v>
       </c>
       <c r="D54" s="1"/>
       <c r="E54" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2367,14 +2384,14 @@
         <v>28</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C56" s="1">
         <v>1</v>
       </c>
       <c r="D56" s="1"/>
       <c r="E56" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2382,14 +2399,14 @@
         <v>28</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C57" s="1">
         <v>1</v>
       </c>
       <c r="D57" s="1"/>
       <c r="E57" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="102" x14ac:dyDescent="0.2">
@@ -2397,14 +2414,14 @@
         <v>28</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C58" s="1">
         <v>1</v>
       </c>
       <c r="D58" s="1"/>
       <c r="E58" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2412,14 +2429,14 @@
         <v>28</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C59" s="1">
         <v>1</v>
       </c>
       <c r="D59" s="1"/>
       <c r="E59" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2449,7 +2466,7 @@
       </c>
       <c r="D61" s="1"/>
       <c r="E61" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2464,7 +2481,7 @@
       </c>
       <c r="D62" s="1"/>
       <c r="E62" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2479,7 +2496,7 @@
       </c>
       <c r="D63" s="1"/>
       <c r="E63" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2494,7 +2511,7 @@
       </c>
       <c r="D64" s="1"/>
       <c r="E64" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2502,7 +2519,7 @@
         <v>28</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C65" s="1">
         <v>1</v>
@@ -2511,7 +2528,7 @@
         <v>22</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
@@ -2519,14 +2536,14 @@
         <v>28</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C66" s="1">
         <v>1</v>
       </c>
       <c r="D66" s="1"/>
       <c r="E66" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2540,10 +2557,10 @@
         <v>1</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2551,16 +2568,16 @@
         <v>82</v>
       </c>
       <c r="B68" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C68" s="1">
+        <v>1</v>
+      </c>
+      <c r="D68" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C68" s="1">
-        <v>1</v>
-      </c>
-      <c r="D68" s="1" t="s">
+      <c r="E68" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2568,16 +2585,16 @@
         <v>82</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C69" s="1">
         <v>1</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2592,7 +2609,7 @@
       </c>
       <c r="D70" s="1"/>
       <c r="E70" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2600,14 +2617,14 @@
         <v>28</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C71" s="1">
         <v>1</v>
       </c>
       <c r="D71" s="1"/>
       <c r="E71" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2615,14 +2632,14 @@
         <v>28</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C72" s="1">
         <v>1</v>
       </c>
       <c r="D72" s="1"/>
       <c r="E72" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2630,14 +2647,14 @@
         <v>28</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C73" s="1">
         <v>1</v>
       </c>
       <c r="D73" s="1"/>
       <c r="E73" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2645,14 +2662,14 @@
         <v>28</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C74" s="1">
         <v>1</v>
       </c>
       <c r="D74" s="1"/>
       <c r="E74" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2660,14 +2677,14 @@
         <v>28</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C75" s="1">
         <v>1</v>
       </c>
       <c r="D75" s="1"/>
       <c r="E75" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2675,14 +2692,14 @@
         <v>28</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C76" s="1">
         <v>1</v>
       </c>
       <c r="D76" s="1"/>
       <c r="E76" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2702,7 +2719,7 @@
     </row>
     <row r="78" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>42</v>
@@ -2720,14 +2737,14 @@
         <v>28</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C79" s="1">
         <v>1</v>
       </c>
       <c r="D79" s="1"/>
       <c r="E79" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2742,7 +2759,7 @@
       </c>
       <c r="D80" s="1"/>
       <c r="E80" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2750,16 +2767,16 @@
         <v>28</v>
       </c>
       <c r="B81" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C81" s="1">
+        <v>1</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E81" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="C81" s="1">
-        <v>1</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="E81" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2767,14 +2784,14 @@
         <v>28</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C82" s="1">
         <v>1</v>
       </c>
       <c r="D82" s="1"/>
       <c r="E82" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2782,14 +2799,14 @@
         <v>28</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C83" s="1">
         <v>1</v>
       </c>
       <c r="D83" s="1"/>
       <c r="E83" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="153" x14ac:dyDescent="0.2">
@@ -2797,19 +2814,19 @@
         <v>28</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C84" s="1">
         <v>1</v>
       </c>
       <c r="D84" s="1"/>
       <c r="E84" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>46</v>
@@ -2827,14 +2844,14 @@
         <v>28</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C86" s="1">
         <v>1</v>
       </c>
       <c r="D86" s="1"/>
       <c r="E86" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -2842,14 +2859,14 @@
         <v>28</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C87" s="1">
         <v>1</v>
       </c>
       <c r="D87" s="1"/>
       <c r="E87" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
@@ -2857,14 +2874,14 @@
         <v>28</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C88" s="1">
         <v>1</v>
       </c>
       <c r="D88" s="1"/>
       <c r="E88" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -2872,14 +2889,14 @@
         <v>28</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C89" s="1">
         <v>1</v>
       </c>
       <c r="D89" s="1"/>
       <c r="E89" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -2887,14 +2904,14 @@
         <v>28</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C90" s="1">
         <v>1</v>
       </c>
       <c r="D90" s="1"/>
       <c r="E90" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -2902,14 +2919,14 @@
         <v>28</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C91" s="1">
         <v>1</v>
       </c>
       <c r="D91" s="1"/>
       <c r="E91" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2917,16 +2934,16 @@
         <v>28</v>
       </c>
       <c r="B92" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C92" s="1">
+        <v>1</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="C92" s="1">
-        <v>1</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2940,7 +2957,7 @@
         <v>1</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>78</v>
@@ -2951,14 +2968,16 @@
         <v>84</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>87</v>
+        <v>327</v>
       </c>
       <c r="C94" s="1">
         <v>1</v>
       </c>
-      <c r="D94" s="1"/>
+      <c r="D94" s="1" t="s">
+        <v>330</v>
+      </c>
       <c r="E94" s="2" t="s">
-        <v>86</v>
+        <v>328</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2966,44 +2985,48 @@
         <v>84</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C95" s="1">
         <v>1</v>
       </c>
-      <c r="D95" s="1"/>
+      <c r="D95" s="1" t="s">
+        <v>331</v>
+      </c>
       <c r="E95" s="2" t="s">
-        <v>89</v>
+        <v>329</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C96" s="1">
+        <v>1</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B97" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C96" s="1">
-        <v>1</v>
-      </c>
-      <c r="D96" s="1"/>
-      <c r="E96" s="2" t="s">
+      <c r="C97" s="1">
+        <v>1</v>
+      </c>
+      <c r="D97" s="1"/>
+      <c r="E97" s="2" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A97" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="C97" s="1">
-        <v>1</v>
-      </c>
-      <c r="D97" s="1"/>
-      <c r="E97" s="1" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
@@ -3011,187 +3034,187 @@
         <v>28</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C98" s="1">
         <v>1</v>
       </c>
       <c r="D98" s="1"/>
       <c r="E98" s="1" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>96</v>
+        <v>28</v>
       </c>
       <c r="B99" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C99" s="1">
+        <v>1</v>
+      </c>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C99" s="1">
-        <v>1</v>
-      </c>
-      <c r="D99" s="1" t="s">
+      <c r="C100" s="1">
+        <v>1</v>
+      </c>
+      <c r="D100" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E99" s="2" t="s">
+      <c r="E100" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="102" x14ac:dyDescent="0.2">
-      <c r="A100" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C100" s="1">
-        <v>1</v>
-      </c>
-      <c r="D100" s="1"/>
-      <c r="E100" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:5" ht="102" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>25</v>
+        <v>171</v>
       </c>
       <c r="C101" s="1">
         <v>1</v>
       </c>
       <c r="D101" s="1"/>
       <c r="E101" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B102" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C102" s="1">
+        <v>1</v>
+      </c>
+      <c r="D102" s="1"/>
+      <c r="E102" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C103" s="1">
+        <v>1</v>
+      </c>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="C102" s="1">
-        <v>1</v>
-      </c>
-      <c r="D102" s="1"/>
-      <c r="E102" s="1" t="s">
+    </row>
+    <row r="104" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C104" s="1">
+        <v>1</v>
+      </c>
+      <c r="D104" s="1"/>
+      <c r="E104" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B105" s="1" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A103" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="C103" s="1">
-        <v>1</v>
-      </c>
-      <c r="D103" s="1"/>
-      <c r="E103" s="2" t="s">
+      <c r="C105" s="1">
+        <v>1</v>
+      </c>
+      <c r="D105" s="1"/>
+      <c r="E105" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C106" s="1">
+        <v>1</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C107" s="1">
+        <v>1</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C108" s="1">
+        <v>1</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C109" s="1">
+        <v>1</v>
+      </c>
+      <c r="D109" s="1"/>
+      <c r="E109" s="2" t="s">
         <v>312</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A104" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="C104" s="1">
-        <v>1</v>
-      </c>
-      <c r="D104" s="1"/>
-      <c r="E104" s="1" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A105" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C105" s="1">
-        <v>1</v>
-      </c>
-      <c r="D105" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E105" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A106" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C106" s="1">
-        <v>1</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A107" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C107" s="1">
-        <v>1</v>
-      </c>
-      <c r="D107" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E107" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A108" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B108" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C108" s="1">
-        <v>1</v>
-      </c>
-      <c r="D108" s="1"/>
-      <c r="E108" s="2" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A109" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B109" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="C109" s="1">
-        <v>1</v>
-      </c>
-      <c r="D109" s="1"/>
-      <c r="E109" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
@@ -3199,29 +3222,29 @@
         <v>28</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C110" s="1">
         <v>1</v>
       </c>
       <c r="D110" s="1"/>
       <c r="E110" s="1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="C111" s="1">
         <v>1</v>
       </c>
       <c r="D111" s="1"/>
-      <c r="E111" s="2" t="s">
-        <v>270</v>
+      <c r="E111" s="1" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -3229,121 +3252,123 @@
         <v>28</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>142</v>
+        <v>268</v>
       </c>
       <c r="C112" s="1">
         <v>1</v>
       </c>
-      <c r="D112" s="1"/>
+      <c r="D112" s="1" t="s">
+        <v>191</v>
+      </c>
       <c r="E112" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C113" s="1">
         <v>1</v>
       </c>
       <c r="D113" s="1"/>
       <c r="E113" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>216</v>
+        <v>143</v>
       </c>
       <c r="C114" s="1">
         <v>1</v>
       </c>
-      <c r="D114" s="1" t="s">
-        <v>217</v>
-      </c>
+      <c r="D114" s="1"/>
       <c r="E114" s="2" t="s">
-        <v>220</v>
+        <v>144</v>
       </c>
     </row>
     <row r="115" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>26</v>
+        <v>215</v>
       </c>
       <c r="C115" s="1">
         <v>1</v>
       </c>
-      <c r="D115" s="1"/>
+      <c r="D115" s="1" t="s">
+        <v>216</v>
+      </c>
       <c r="E115" s="2" t="s">
-        <v>314</v>
+        <v>219</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="C116" s="1">
         <v>1</v>
       </c>
       <c r="D116" s="1"/>
       <c r="E116" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>198</v>
+        <v>75</v>
       </c>
       <c r="C117" s="1">
         <v>1</v>
       </c>
       <c r="D117" s="1"/>
       <c r="E117" s="2" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C118" s="1">
+        <v>1</v>
+      </c>
+      <c r="D118" s="1"/>
+      <c r="E118" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B118" s="1" t="s">
+      <c r="B119" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C118" s="1">
-        <v>1</v>
-      </c>
-      <c r="D118" s="1"/>
-      <c r="E118" s="1" t="s">
+      <c r="C119" s="1">
+        <v>1</v>
+      </c>
+      <c r="D119" s="1"/>
+      <c r="E119" s="1" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A119" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C119" s="1">
-        <v>1</v>
-      </c>
-      <c r="D119" s="1"/>
-      <c r="E119" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="120" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -3351,125 +3376,125 @@
         <v>28</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>146</v>
+        <v>36</v>
       </c>
       <c r="C120" s="1">
         <v>1</v>
       </c>
-      <c r="D120" s="1" t="s">
-        <v>129</v>
-      </c>
+      <c r="D120" s="1"/>
       <c r="E120" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>96</v>
+        <v>28</v>
       </c>
       <c r="B121" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C121" s="1">
+        <v>1</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A122" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B122" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C121" s="1">
-        <v>1</v>
-      </c>
-      <c r="D121" s="1" t="s">
+      <c r="C122" s="1">
+        <v>1</v>
+      </c>
+      <c r="D122" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E121" s="2" t="s">
+      <c r="E122" s="2" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A122" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B122" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C122" s="1">
-        <v>1</v>
-      </c>
-      <c r="D122" s="1"/>
-      <c r="E122" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="123" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C123" s="1">
+        <v>1</v>
+      </c>
+      <c r="D123" s="1"/>
+      <c r="E123" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A124" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B123" s="1" t="s">
+      <c r="B124" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C124" s="1">
+        <v>1</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E124" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C123" s="1">
-        <v>1</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="E123" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A124" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B124" s="1" t="s">
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C125" s="1">
+        <v>1</v>
+      </c>
+      <c r="D125" s="1"/>
+      <c r="E125" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="C124" s="1">
-        <v>1</v>
-      </c>
-      <c r="D124" s="1"/>
-      <c r="E124" s="1" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A125" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="C125" s="1">
-        <v>1</v>
-      </c>
-      <c r="D125" s="1"/>
-      <c r="E125" s="2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    </row>
+    <row r="126" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>177</v>
+        <v>203</v>
       </c>
       <c r="C126" s="1">
         <v>1</v>
       </c>
       <c r="D126" s="1"/>
       <c r="E126" s="2" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>147</v>
+        <v>176</v>
       </c>
       <c r="C127" s="1">
         <v>1</v>
       </c>
       <c r="D127" s="1"/>
       <c r="E127" s="2" t="s">
-        <v>148</v>
+        <v>316</v>
       </c>
     </row>
     <row r="128" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -3477,59 +3502,59 @@
         <v>28</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>196</v>
+        <v>146</v>
       </c>
       <c r="C128" s="1">
         <v>1</v>
       </c>
       <c r="D128" s="1"/>
       <c r="E128" s="2" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B129" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C129" s="1">
+        <v>1</v>
+      </c>
+      <c r="D129" s="1"/>
+      <c r="E129" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C130" s="1">
+        <v>1</v>
+      </c>
+      <c r="D130" s="1"/>
+      <c r="E130" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="C129" s="1">
-        <v>1</v>
-      </c>
-      <c r="D129" s="1"/>
-      <c r="E129" s="1" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="130" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A130" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B130" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="C130" s="1">
-        <v>1</v>
-      </c>
-      <c r="D130" s="1"/>
-      <c r="E130" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="131" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    </row>
+    <row r="131" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C131" s="1">
         <v>1</v>
       </c>
       <c r="D131" s="1"/>
       <c r="E131" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="132" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -3537,269 +3562,269 @@
         <v>28</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="C132" s="1">
         <v>1</v>
       </c>
       <c r="D132" s="1"/>
       <c r="E132" s="2" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="133" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="C133" s="1">
         <v>1</v>
       </c>
       <c r="D133" s="1"/>
       <c r="E133" s="2" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="134" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="C134" s="1">
         <v>1</v>
       </c>
       <c r="D134" s="1"/>
       <c r="E134" s="2" t="s">
-        <v>154</v>
+        <v>319</v>
       </c>
     </row>
     <row r="135" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>30</v>
+        <v>152</v>
       </c>
       <c r="C135" s="1">
         <v>1</v>
       </c>
       <c r="D135" s="1"/>
       <c r="E135" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="136" spans="1:5" ht="85" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>183</v>
+        <v>30</v>
       </c>
       <c r="C136" s="1">
         <v>1</v>
       </c>
       <c r="D136" s="1"/>
       <c r="E136" s="2" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="137" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" ht="85" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>32</v>
+        <v>182</v>
       </c>
       <c r="C137" s="1">
         <v>1</v>
       </c>
       <c r="D137" s="1"/>
       <c r="E137" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="138" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>105</v>
+        <v>32</v>
       </c>
       <c r="C138" s="1">
         <v>1</v>
       </c>
       <c r="D138" s="1"/>
       <c r="E138" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="139" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C139" s="1">
         <v>1</v>
       </c>
       <c r="D139" s="1"/>
       <c r="E139" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C140" s="1">
+        <v>1</v>
+      </c>
+      <c r="D140" s="1"/>
+      <c r="E140" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A141" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B140" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="C140" s="1">
-        <v>1</v>
-      </c>
-      <c r="D140" s="1"/>
-      <c r="E140" s="2"/>
-    </row>
-    <row r="141" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A141" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="B141" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C141" s="1">
+        <v>1</v>
+      </c>
+      <c r="D141" s="1"/>
+      <c r="E141" s="2"/>
+    </row>
+    <row r="142" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A142" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C142" s="1">
+        <v>1</v>
+      </c>
+      <c r="D142" s="1"/>
+      <c r="E142" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C141" s="1">
-        <v>1</v>
-      </c>
-      <c r="D141" s="1"/>
-      <c r="E141" s="2" t="s">
+    </row>
+    <row r="143" spans="1:5" ht="85" x14ac:dyDescent="0.2">
+      <c r="A143" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C143" s="1">
+        <v>1</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A144" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B144" s="1" t="s">
         <v>156</v>
-      </c>
-    </row>
-    <row r="142" spans="1:5" ht="85" x14ac:dyDescent="0.2">
-      <c r="A142" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B142" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C142" s="1">
-        <v>1</v>
-      </c>
-      <c r="D142" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E142" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="143" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A143" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B143" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C143" s="1">
-        <v>1</v>
-      </c>
-      <c r="D143" s="1"/>
-      <c r="E143" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="144" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A144" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B144" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C144" s="1">
         <v>1</v>
       </c>
       <c r="D144" s="1"/>
       <c r="E144" s="2" t="s">
-        <v>210</v>
+        <v>157</v>
       </c>
     </row>
     <row r="145" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>180</v>
+        <v>47</v>
       </c>
       <c r="C145" s="1">
         <v>1</v>
       </c>
       <c r="D145" s="1"/>
       <c r="E145" s="2" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="146" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>37</v>
+        <v>179</v>
       </c>
       <c r="C146" s="1">
         <v>1</v>
       </c>
       <c r="D146" s="1"/>
       <c r="E146" s="2" t="s">
-        <v>40</v>
+        <v>321</v>
       </c>
     </row>
     <row r="147" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="C147" s="1">
         <v>1</v>
       </c>
       <c r="D147" s="1"/>
       <c r="E147" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A148" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C148" s="1">
+        <v>1</v>
+      </c>
+      <c r="D148" s="1"/>
+      <c r="E148" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A148" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B148" s="1" t="s">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A149" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C149" s="1">
+        <v>1</v>
+      </c>
+      <c r="D149" s="1"/>
+      <c r="E149" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="C148" s="1">
-        <v>1</v>
-      </c>
-      <c r="D148" s="1"/>
-      <c r="E148" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="149" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A149" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B149" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C149" s="1">
-        <v>1</v>
-      </c>
-      <c r="D149" s="1"/>
-      <c r="E149" s="2" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="150" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -3807,135 +3832,150 @@
         <v>28</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>178</v>
+        <v>27</v>
       </c>
       <c r="C150" s="1">
         <v>1</v>
       </c>
       <c r="D150" s="1"/>
       <c r="E150" s="2" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="151" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C151" s="1">
+        <v>1</v>
+      </c>
+      <c r="D151" s="1"/>
+      <c r="E151" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A152" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B151" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C151" s="1">
-        <v>1</v>
-      </c>
-      <c r="D151" s="1" t="s">
+      <c r="B152" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E151" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A152" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B152" s="1" t="s">
+      <c r="C152" s="1">
+        <v>1</v>
+      </c>
+      <c r="D152" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A153" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C153" s="1">
+        <v>1</v>
+      </c>
+      <c r="D153" s="1"/>
+      <c r="E153" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C152" s="1">
-        <v>1</v>
-      </c>
-      <c r="D152" s="1"/>
-      <c r="E152" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="153" spans="1:5" ht="85" x14ac:dyDescent="0.2">
-      <c r="A153" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B153" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C153" s="1">
-        <v>1</v>
-      </c>
-      <c r="D153" s="1"/>
-      <c r="E153" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="154" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    </row>
+    <row r="154" spans="1:5" ht="85" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C154" s="1">
         <v>1</v>
       </c>
       <c r="D154" s="1"/>
       <c r="E154" s="2" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B155" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C155" s="1">
+        <v>1</v>
+      </c>
+      <c r="D155" s="1"/>
+      <c r="E155" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A156" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C156" s="1">
+        <v>1</v>
+      </c>
+      <c r="D156" s="1"/>
+      <c r="E156" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="C155" s="1">
-        <v>1</v>
-      </c>
-      <c r="D155" s="1"/>
-      <c r="E155" s="1" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="156" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A156" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B156" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="C156" s="1">
-        <v>1</v>
-      </c>
-      <c r="D156" s="1"/>
-      <c r="E156" s="2" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="157" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="C157" s="1">
         <v>1</v>
       </c>
       <c r="D157" s="1"/>
       <c r="E157" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="158" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>10</v>
+        <v>196</v>
       </c>
       <c r="C158" s="1">
         <v>1</v>
       </c>
       <c r="D158" s="1"/>
       <c r="E158" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A159" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C159" s="1">
+        <v>1</v>
+      </c>
+      <c r="D159" s="1"/>
+      <c r="E159" s="2" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>